<commit_message>
Calendario estrategico completo (nov e dez) e cronograma de seis meses em formato de calendario
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/08-calendario-estrategico.xlsx
+++ b/08-calendario-estrategico.xlsx
@@ -17,8 +17,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -168,7 +169,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -229,6 +230,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -716,7 +726,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K51"/>
+  <dimension ref="A1:K59"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="16" min="1" max="1"/>
@@ -742,7 +752,7 @@
     <row r="2" ht="15" customHeight="1" s="16">
       <c r="A2" s="15" t="inlineStr">
         <is>
-          <t>Pousada Vila Mathilde: novembro de 2026 (4 semanas). Depois, repetir o ciclo e duplicar a aba.</t>
+          <t>Pousada Vila Mathilde: novembro e dezembro de 2026 (9 semanas). Depois, repetir o ciclo e duplicar a aba.</t>
         </is>
       </c>
     </row>
@@ -2099,305 +2109,1468 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="56" customHeight="1" s="16">
-      <c r="A29" s="2" t="n"/>
-      <c r="B29" s="3" t="n"/>
-      <c r="C29" s="3" t="n"/>
-      <c r="D29" s="3" t="n"/>
-      <c r="E29" s="3" t="n"/>
-      <c r="F29" s="4" t="n"/>
-      <c r="G29" s="4" t="n"/>
-      <c r="H29" s="4" t="n"/>
-      <c r="I29" s="3" t="n"/>
-      <c r="J29" s="5" t="n"/>
-      <c r="K29" s="4" t="n"/>
-    </row>
-    <row r="30" ht="56" customHeight="1" s="16">
-      <c r="A30" s="2" t="n"/>
-      <c r="B30" s="3" t="n"/>
-      <c r="C30" s="3" t="n"/>
-      <c r="D30" s="3" t="n"/>
-      <c r="E30" s="3" t="n"/>
-      <c r="F30" s="4" t="n"/>
-      <c r="G30" s="4" t="n"/>
-      <c r="H30" s="4" t="n"/>
-      <c r="I30" s="3" t="n"/>
-      <c r="J30" s="5" t="n"/>
-      <c r="K30" s="4" t="n"/>
-    </row>
-    <row r="31" ht="56" customHeight="1" s="16">
-      <c r="A31" s="2" t="n"/>
-      <c r="B31" s="3" t="n"/>
-      <c r="C31" s="3" t="n"/>
-      <c r="D31" s="3" t="n"/>
-      <c r="E31" s="3" t="n"/>
-      <c r="F31" s="4" t="n"/>
-      <c r="G31" s="4" t="n"/>
-      <c r="H31" s="4" t="n"/>
-      <c r="I31" s="3" t="n"/>
-      <c r="J31" s="5" t="n"/>
-      <c r="K31" s="4" t="n"/>
-    </row>
-    <row r="32" ht="56" customHeight="1" s="16">
-      <c r="A32" s="2" t="n"/>
-      <c r="B32" s="3" t="n"/>
-      <c r="C32" s="3" t="n"/>
-      <c r="D32" s="3" t="n"/>
-      <c r="E32" s="3" t="n"/>
-      <c r="F32" s="4" t="n"/>
-      <c r="G32" s="4" t="n"/>
-      <c r="H32" s="4" t="n"/>
-      <c r="I32" s="3" t="n"/>
-      <c r="J32" s="5" t="n"/>
-      <c r="K32" s="4" t="n"/>
-    </row>
-    <row r="33" ht="56" customHeight="1" s="16">
-      <c r="A33" s="2" t="n"/>
-      <c r="B33" s="3" t="n"/>
-      <c r="C33" s="3" t="n"/>
-      <c r="D33" s="3" t="n"/>
-      <c r="E33" s="3" t="n"/>
-      <c r="F33" s="4" t="n"/>
-      <c r="G33" s="4" t="n"/>
-      <c r="H33" s="4" t="n"/>
-      <c r="I33" s="3" t="n"/>
-      <c r="J33" s="5" t="n"/>
-      <c r="K33" s="4" t="n"/>
-    </row>
-    <row r="34" ht="56" customHeight="1" s="16">
-      <c r="A34" s="2" t="n"/>
-      <c r="B34" s="3" t="n"/>
-      <c r="C34" s="3" t="n"/>
-      <c r="D34" s="3" t="n"/>
-      <c r="E34" s="3" t="n"/>
-      <c r="F34" s="4" t="n"/>
-      <c r="G34" s="4" t="n"/>
-      <c r="H34" s="4" t="n"/>
-      <c r="I34" s="3" t="n"/>
-      <c r="J34" s="5" t="n"/>
-      <c r="K34" s="4" t="n"/>
-    </row>
-    <row r="35" ht="56" customHeight="1" s="16">
-      <c r="A35" s="2" t="n"/>
-      <c r="B35" s="3" t="n"/>
-      <c r="C35" s="3" t="n"/>
-      <c r="D35" s="3" t="n"/>
-      <c r="E35" s="3" t="n"/>
-      <c r="F35" s="4" t="n"/>
-      <c r="G35" s="4" t="n"/>
-      <c r="H35" s="4" t="n"/>
-      <c r="I35" s="3" t="n"/>
-      <c r="J35" s="5" t="n"/>
-      <c r="K35" s="4" t="n"/>
-    </row>
-    <row r="36" ht="56" customHeight="1" s="16">
-      <c r="A36" s="2" t="n"/>
-      <c r="B36" s="3" t="n"/>
-      <c r="C36" s="3" t="n"/>
-      <c r="D36" s="3" t="n"/>
-      <c r="E36" s="3" t="n"/>
-      <c r="F36" s="4" t="n"/>
-      <c r="G36" s="4" t="n"/>
-      <c r="H36" s="4" t="n"/>
-      <c r="I36" s="3" t="n"/>
-      <c r="J36" s="5" t="n"/>
-      <c r="K36" s="4" t="n"/>
-    </row>
-    <row r="37" ht="56" customHeight="1" s="16">
-      <c r="A37" s="2" t="n"/>
-      <c r="B37" s="3" t="n"/>
-      <c r="C37" s="3" t="n"/>
-      <c r="D37" s="3" t="n"/>
-      <c r="E37" s="3" t="n"/>
-      <c r="F37" s="4" t="n"/>
-      <c r="G37" s="4" t="n"/>
-      <c r="H37" s="4" t="n"/>
-      <c r="I37" s="3" t="n"/>
-      <c r="J37" s="5" t="n"/>
-      <c r="K37" s="4" t="n"/>
-    </row>
-    <row r="38" ht="56" customHeight="1" s="16">
-      <c r="A38" s="2" t="n"/>
-      <c r="B38" s="3" t="n"/>
-      <c r="C38" s="3" t="n"/>
-      <c r="D38" s="3" t="n"/>
-      <c r="E38" s="3" t="n"/>
-      <c r="F38" s="4" t="n"/>
-      <c r="G38" s="4" t="n"/>
-      <c r="H38" s="4" t="n"/>
-      <c r="I38" s="3" t="n"/>
-      <c r="J38" s="5" t="n"/>
-      <c r="K38" s="4" t="n"/>
-    </row>
-    <row r="39" ht="56" customHeight="1" s="16">
-      <c r="A39" s="2" t="n"/>
-      <c r="B39" s="3" t="n"/>
-      <c r="C39" s="3" t="n"/>
-      <c r="D39" s="3" t="n"/>
-      <c r="E39" s="3" t="n"/>
-      <c r="F39" s="4" t="n"/>
-      <c r="G39" s="4" t="n"/>
-      <c r="H39" s="4" t="n"/>
-      <c r="I39" s="3" t="n"/>
-      <c r="J39" s="5" t="n"/>
-      <c r="K39" s="4" t="n"/>
-    </row>
-    <row r="40" ht="56" customHeight="1" s="16">
-      <c r="A40" s="2" t="n"/>
-      <c r="B40" s="3" t="n"/>
-      <c r="C40" s="3" t="n"/>
-      <c r="D40" s="3" t="n"/>
-      <c r="E40" s="3" t="n"/>
-      <c r="F40" s="4" t="n"/>
-      <c r="G40" s="4" t="n"/>
-      <c r="H40" s="4" t="n"/>
-      <c r="I40" s="3" t="n"/>
-      <c r="J40" s="5" t="n"/>
-      <c r="K40" s="4" t="n"/>
-    </row>
-    <row r="41" ht="56" customHeight="1" s="16">
-      <c r="A41" s="2" t="n"/>
-      <c r="B41" s="3" t="n"/>
-      <c r="C41" s="3" t="n"/>
-      <c r="D41" s="3" t="n"/>
-      <c r="E41" s="3" t="n"/>
-      <c r="F41" s="4" t="n"/>
-      <c r="G41" s="4" t="n"/>
-      <c r="H41" s="4" t="n"/>
-      <c r="I41" s="3" t="n"/>
-      <c r="J41" s="5" t="n"/>
-      <c r="K41" s="4" t="n"/>
-    </row>
-    <row r="42" ht="56" customHeight="1" s="16">
-      <c r="A42" s="2" t="n"/>
-      <c r="B42" s="3" t="n"/>
-      <c r="C42" s="3" t="n"/>
-      <c r="D42" s="3" t="n"/>
-      <c r="E42" s="3" t="n"/>
-      <c r="F42" s="4" t="n"/>
-      <c r="G42" s="4" t="n"/>
-      <c r="H42" s="4" t="n"/>
-      <c r="I42" s="3" t="n"/>
-      <c r="J42" s="5" t="n"/>
-      <c r="K42" s="4" t="n"/>
-    </row>
-    <row r="43" ht="56" customHeight="1" s="16">
-      <c r="A43" s="2" t="n"/>
-      <c r="B43" s="3" t="n"/>
-      <c r="C43" s="3" t="n"/>
-      <c r="D43" s="3" t="n"/>
-      <c r="E43" s="3" t="n"/>
-      <c r="F43" s="4" t="n"/>
-      <c r="G43" s="4" t="n"/>
-      <c r="H43" s="4" t="n"/>
-      <c r="I43" s="3" t="n"/>
-      <c r="J43" s="5" t="n"/>
-      <c r="K43" s="4" t="n"/>
-    </row>
-    <row r="44" ht="56" customHeight="1" s="16">
-      <c r="A44" s="2" t="n"/>
-      <c r="B44" s="3" t="n"/>
-      <c r="C44" s="3" t="n"/>
-      <c r="D44" s="3" t="n"/>
-      <c r="E44" s="3" t="n"/>
-      <c r="F44" s="4" t="n"/>
-      <c r="G44" s="4" t="n"/>
-      <c r="H44" s="4" t="n"/>
-      <c r="I44" s="3" t="n"/>
-      <c r="J44" s="5" t="n"/>
-      <c r="K44" s="4" t="n"/>
-    </row>
-    <row r="45" ht="56" customHeight="1" s="16">
-      <c r="A45" s="2" t="n"/>
-      <c r="B45" s="3" t="n"/>
-      <c r="C45" s="3" t="n"/>
-      <c r="D45" s="3" t="n"/>
-      <c r="E45" s="3" t="n"/>
-      <c r="F45" s="4" t="n"/>
-      <c r="G45" s="4" t="n"/>
-      <c r="H45" s="4" t="n"/>
-      <c r="I45" s="3" t="n"/>
-      <c r="J45" s="5" t="n"/>
-      <c r="K45" s="4" t="n"/>
-    </row>
-    <row r="46" ht="56" customHeight="1" s="16">
-      <c r="A46" s="2" t="n"/>
-      <c r="B46" s="3" t="n"/>
-      <c r="C46" s="3" t="n"/>
-      <c r="D46" s="3" t="n"/>
-      <c r="E46" s="3" t="n"/>
-      <c r="F46" s="4" t="n"/>
-      <c r="G46" s="4" t="n"/>
-      <c r="H46" s="4" t="n"/>
-      <c r="I46" s="3" t="n"/>
-      <c r="J46" s="5" t="n"/>
-      <c r="K46" s="4" t="n"/>
-    </row>
-    <row r="47" ht="56" customHeight="1" s="16">
-      <c r="A47" s="2" t="n"/>
-      <c r="B47" s="3" t="n"/>
-      <c r="C47" s="3" t="n"/>
-      <c r="D47" s="3" t="n"/>
-      <c r="E47" s="3" t="n"/>
-      <c r="F47" s="4" t="n"/>
-      <c r="G47" s="4" t="n"/>
-      <c r="H47" s="4" t="n"/>
-      <c r="I47" s="3" t="n"/>
-      <c r="J47" s="5" t="n"/>
-      <c r="K47" s="4" t="n"/>
-    </row>
-    <row r="48" ht="56" customHeight="1" s="16">
-      <c r="A48" s="2" t="n"/>
-      <c r="B48" s="3" t="n"/>
-      <c r="C48" s="3" t="n"/>
-      <c r="D48" s="3" t="n"/>
-      <c r="E48" s="3" t="n"/>
-      <c r="F48" s="4" t="n"/>
-      <c r="G48" s="4" t="n"/>
-      <c r="H48" s="4" t="n"/>
-      <c r="I48" s="3" t="n"/>
-      <c r="J48" s="5" t="n"/>
-      <c r="K48" s="4" t="n"/>
-    </row>
-    <row r="49" ht="56" customHeight="1" s="16">
-      <c r="A49" s="2" t="n"/>
-      <c r="B49" s="3" t="n"/>
-      <c r="C49" s="3" t="n"/>
-      <c r="D49" s="3" t="n"/>
-      <c r="E49" s="3" t="n"/>
-      <c r="F49" s="4" t="n"/>
-      <c r="G49" s="4" t="n"/>
-      <c r="H49" s="4" t="n"/>
-      <c r="I49" s="3" t="n"/>
-      <c r="J49" s="5" t="n"/>
-      <c r="K49" s="4" t="n"/>
-    </row>
-    <row r="50" ht="56" customHeight="1" s="16">
-      <c r="A50" s="2" t="n"/>
-      <c r="B50" s="3" t="n"/>
-      <c r="C50" s="3" t="n"/>
-      <c r="D50" s="3" t="n"/>
-      <c r="E50" s="3" t="n"/>
-      <c r="F50" s="4" t="n"/>
-      <c r="G50" s="4" t="n"/>
-      <c r="H50" s="4" t="n"/>
-      <c r="I50" s="3" t="n"/>
-      <c r="J50" s="5" t="n"/>
-      <c r="K50" s="4" t="n"/>
-    </row>
-    <row r="51" ht="56" customHeight="1" s="16">
-      <c r="A51" s="2" t="n"/>
-      <c r="B51" s="3" t="n"/>
-      <c r="C51" s="3" t="n"/>
-      <c r="D51" s="3" t="n"/>
-      <c r="E51" s="3" t="n"/>
-      <c r="F51" s="4" t="n"/>
-      <c r="G51" s="4" t="n"/>
-      <c r="H51" s="4" t="n"/>
-      <c r="I51" s="3" t="n"/>
-      <c r="J51" s="5" t="n"/>
-      <c r="K51" s="4" t="n"/>
-    </row>
+    <row r="29" ht="78" customHeight="1" s="16">
+      <c r="A29" s="22" t="n">
+        <v>46356</v>
+      </c>
+      <c r="B29" s="23">
+        <f>TEXT(A29,"dddd")</f>
+        <v/>
+      </c>
+      <c r="C29" s="23" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="D29" s="23" t="inlineStr">
+        <is>
+          <t>Reels</t>
+        </is>
+      </c>
+      <c r="E29" s="23" t="inlineStr">
+        <is>
+          <t>Bastidores</t>
+        </is>
+      </c>
+      <c r="F29" s="23" t="inlineStr">
+        <is>
+          <t>Preparando o café</t>
+        </is>
+      </c>
+      <c r="G29" s="23" t="inlineStr">
+        <is>
+          <t>Antes de você acordar, o café já está sendo feito. Pão, bolo e fruta fresca para começar bem o dia.</t>
+        </is>
+      </c>
+      <c r="H29" s="23" t="inlineStr">
+        <is>
+          <t>#CafeDaRoca #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+        </is>
+      </c>
+      <c r="I29" s="23" t="inlineStr">
+        <is>
+          <t>Dono</t>
+        </is>
+      </c>
+      <c r="J29" s="26" t="inlineStr">
+        <is>
+          <t>Ideia</t>
+        </is>
+      </c>
+      <c r="K29" s="23" t="inlineStr">
+        <is>
+          <t>Gravar o preparo do café logo cedo, de 20 segundos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="78" customHeight="1" s="16">
+      <c r="A30" s="22" t="n">
+        <v>46357</v>
+      </c>
+      <c r="B30" s="23">
+        <f>TEXT(A30,"dddd")</f>
+        <v/>
+      </c>
+      <c r="C30" s="23" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="D30" s="23" t="inlineStr">
+        <is>
+          <t>Vídeo curto</t>
+        </is>
+      </c>
+      <c r="E30" s="23" t="inlineStr">
+        <is>
+          <t>Experiência</t>
+        </is>
+      </c>
+      <c r="F30" s="23" t="inlineStr">
+        <is>
+          <t>Presente na chegada</t>
+        </is>
+      </c>
+      <c r="G30" s="23" t="inlineStr">
+        <is>
+          <t>Quem chega leva uma lembrança: uma caneca ou mini cesta com um bilhete com o seu nome.</t>
+        </is>
+      </c>
+      <c r="H30" s="23" t="inlineStr">
+        <is>
+          <t>#PresenteDeBoasVindas #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+        </is>
+      </c>
+      <c r="I30" s="23" t="inlineStr">
+        <is>
+          <t>Dono</t>
+        </is>
+      </c>
+      <c r="J30" s="26" t="inlineStr">
+        <is>
+          <t>Ideia</t>
+        </is>
+      </c>
+      <c r="K30" s="23" t="inlineStr">
+        <is>
+          <t>Mostrar o presente sendo entregue, com autorização do hóspede.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="78" customHeight="1" s="16">
+      <c r="A31" s="22" t="n">
+        <v>46358</v>
+      </c>
+      <c r="B31" s="23">
+        <f>TEXT(A31,"dddd")</f>
+        <v/>
+      </c>
+      <c r="C31" s="23" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="D31" s="23" t="inlineStr">
+        <is>
+          <t>Vídeo</t>
+        </is>
+      </c>
+      <c r="E31" s="23" t="inlineStr">
+        <is>
+          <t>História</t>
+        </is>
+      </c>
+      <c r="F31" s="23" t="inlineStr">
+        <is>
+          <t>Matilde nasceu do trem</t>
+        </is>
+      </c>
+      <c r="G31" s="23" t="inlineStr">
+        <is>
+          <t>O nome Mathilde vem da esposa do engenheiro da ferrovia, segundo relatos locais. Venha conhecer a estação de 1910.</t>
+        </is>
+      </c>
+      <c r="H31" s="23" t="inlineStr">
+        <is>
+          <t>#EstacaoDeMatilde #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+        </is>
+      </c>
+      <c r="I31" s="23" t="inlineStr">
+        <is>
+          <t>Dono</t>
+        </is>
+      </c>
+      <c r="J31" s="26" t="inlineStr">
+        <is>
+          <t>Ideia</t>
+        </is>
+      </c>
+      <c r="K31" s="23" t="inlineStr">
+        <is>
+          <t>Tratar o relato como relato local, não como fato comprovado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="78" customHeight="1" s="16">
+      <c r="A32" s="22" t="n">
+        <v>46359</v>
+      </c>
+      <c r="B32" s="23">
+        <f>TEXT(A32,"dddd")</f>
+        <v/>
+      </c>
+      <c r="C32" s="23" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="D32" s="23" t="inlineStr">
+        <is>
+          <t>Reels</t>
+        </is>
+      </c>
+      <c r="E32" s="23" t="inlineStr">
+        <is>
+          <t>Campanha</t>
+        </is>
+      </c>
+      <c r="F32" s="23" t="inlineStr">
+        <is>
+          <t>Dicas de um roteiro de 2 dias</t>
+        </is>
+      </c>
+      <c r="G32" s="23" t="inlineStr">
+        <is>
+          <t>Dia um: cachoeira e mirante. Dia dois: estação e túnel. No meio, o descanso na Vila Mathilde.</t>
+        </is>
+      </c>
+      <c r="H32" s="23" t="inlineStr">
+        <is>
+          <t>#RoteiroDe2Dias #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+        </is>
+      </c>
+      <c r="I32" s="23" t="inlineStr">
+        <is>
+          <t>Dono</t>
+        </is>
+      </c>
+      <c r="J32" s="26" t="inlineStr">
+        <is>
+          <t>Ideia</t>
+        </is>
+      </c>
+      <c r="K32" s="23" t="inlineStr">
+        <is>
+          <t>Reaproveitar o material do criador parceiro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="78" customHeight="1" s="16">
+      <c r="A33" s="22" t="n">
+        <v>46360</v>
+      </c>
+      <c r="B33" s="23">
+        <f>TEXT(A33,"dddd")</f>
+        <v/>
+      </c>
+      <c r="C33" s="23" t="inlineStr">
+        <is>
+          <t>Google Perfil</t>
+        </is>
+      </c>
+      <c r="D33" s="23" t="inlineStr">
+        <is>
+          <t>Post</t>
+        </is>
+      </c>
+      <c r="E33" s="23" t="inlineStr">
+        <is>
+          <t>Campanha</t>
+        </is>
+      </c>
+      <c r="F33" s="23" t="inlineStr">
+        <is>
+          <t>Natal e Réveillon: datas</t>
+        </is>
+      </c>
+      <c r="G33" s="23" t="inlineStr">
+        <is>
+          <t>As datas de fim de ano costumam esgotar. Pergunte pelos quartos livres no WhatsApp.</t>
+        </is>
+      </c>
+      <c r="H33" s="23" t="inlineStr">
+        <is>
+          <t>#VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+        </is>
+      </c>
+      <c r="I33" s="23" t="inlineStr">
+        <is>
+          <t>Dono</t>
+        </is>
+      </c>
+      <c r="J33" s="26" t="inlineStr">
+        <is>
+          <t>Ideia</t>
+        </is>
+      </c>
+      <c r="K33" s="23" t="inlineStr">
+        <is>
+          <t>Escassez honesta, são só 6 quartos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="78" customHeight="1" s="16">
+      <c r="A34" s="22" t="n">
+        <v>46361</v>
+      </c>
+      <c r="B34" s="23">
+        <f>TEXT(A34,"dddd")</f>
+        <v/>
+      </c>
+      <c r="C34" s="23" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="D34" s="23" t="inlineStr">
+        <is>
+          <t>Transmissão</t>
+        </is>
+      </c>
+      <c r="E34" s="23" t="inlineStr">
+        <is>
+          <t>Campanha</t>
+        </is>
+      </c>
+      <c r="F34" s="23" t="inlineStr">
+        <is>
+          <t>Aniversariantes de dezembro</t>
+        </is>
+      </c>
+      <c r="G34" s="23" t="inlineStr">
+        <is>
+          <t>Se o seu aniversário é em dezembro, a gente quer comemorar com você. Responda aqui para saber a condição especial.</t>
+        </is>
+      </c>
+      <c r="H34" s="23" t="inlineStr">
+        <is>
+          <t>#VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+        </is>
+      </c>
+      <c r="I34" s="23" t="inlineStr">
+        <is>
+          <t>Dono</t>
+        </is>
+      </c>
+      <c r="J34" s="26" t="inlineStr">
+        <is>
+          <t>Ideia</t>
+        </is>
+      </c>
+      <c r="K34" s="23" t="inlineStr">
+        <is>
+          <t>Usar só a lista de quem informou a data de aniversário.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="78" customHeight="1" s="16">
+      <c r="A35" s="22" t="n">
+        <v>46363</v>
+      </c>
+      <c r="B35" s="23">
+        <f>TEXT(A35,"dddd")</f>
+        <v/>
+      </c>
+      <c r="C35" s="23" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="D35" s="23" t="inlineStr">
+        <is>
+          <t>Reels</t>
+        </is>
+      </c>
+      <c r="E35" s="23" t="inlineStr">
+        <is>
+          <t>Depoimento</t>
+        </is>
+      </c>
+      <c r="F35" s="23" t="inlineStr">
+        <is>
+          <t>Hóspedes que voltaram</t>
+        </is>
+      </c>
+      <c r="G35" s="23" t="inlineStr">
+        <is>
+          <t>Tem gente que já voltou duas vezes. Obrigado pela confiança, a casa é de vocês.</t>
+        </is>
+      </c>
+      <c r="H35" s="23" t="inlineStr">
+        <is>
+          <t>#Depoimento #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+        </is>
+      </c>
+      <c r="I35" s="23" t="inlineStr">
+        <is>
+          <t>Dono</t>
+        </is>
+      </c>
+      <c r="J35" s="26" t="inlineStr">
+        <is>
+          <t>Ideia</t>
+        </is>
+      </c>
+      <c r="K35" s="23" t="inlineStr">
+        <is>
+          <t>Só com autorização de quem aparece.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="78" customHeight="1" s="16">
+      <c r="A36" s="22" t="n">
+        <v>46364</v>
+      </c>
+      <c r="B36" s="23">
+        <f>TEXT(A36,"dddd")</f>
+        <v/>
+      </c>
+      <c r="C36" s="23" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="D36" s="23" t="inlineStr">
+        <is>
+          <t>Vídeo curto</t>
+        </is>
+      </c>
+      <c r="E36" s="23" t="inlineStr">
+        <is>
+          <t>Destino</t>
+        </is>
+      </c>
+      <c r="F36" s="23" t="inlineStr">
+        <is>
+          <t>A cachoeira cheia depois da chuva</t>
+        </is>
+      </c>
+      <c r="G36" s="23" t="inlineStr">
+        <is>
+          <t>Depois da chuva, a cachoeira de Matilde fica ainda mais forte. Vale a espera.</t>
+        </is>
+      </c>
+      <c r="H36" s="23" t="inlineStr">
+        <is>
+          <t>#CachoeiraDeMatilde #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+        </is>
+      </c>
+      <c r="I36" s="23" t="inlineStr">
+        <is>
+          <t>Dono</t>
+        </is>
+      </c>
+      <c r="J36" s="26" t="inlineStr">
+        <is>
+          <t>Ideia</t>
+        </is>
+      </c>
+      <c r="K36" s="23" t="inlineStr">
+        <is>
+          <t>Gravar em dia seguinte a chuva, com cuidado nas escadas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="78" customHeight="1" s="16">
+      <c r="A37" s="22" t="n">
+        <v>46365</v>
+      </c>
+      <c r="B37" s="23">
+        <f>TEXT(A37,"dddd")</f>
+        <v/>
+      </c>
+      <c r="C37" s="23" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="D37" s="23" t="inlineStr">
+        <is>
+          <t>Vídeo</t>
+        </is>
+      </c>
+      <c r="E37" s="23" t="inlineStr">
+        <is>
+          <t>Experiência</t>
+        </is>
+      </c>
+      <c r="F37" s="23" t="inlineStr">
+        <is>
+          <t>Jardim e passarinhos</t>
+        </is>
+      </c>
+      <c r="G37" s="23" t="inlineStr">
+        <is>
+          <t>Centenas de aves e flores no jardim. Acorde com o canto delas.</t>
+        </is>
+      </c>
+      <c r="H37" s="23" t="inlineStr">
+        <is>
+          <t>#Sossego #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+        </is>
+      </c>
+      <c r="I37" s="23" t="inlineStr">
+        <is>
+          <t>Dono</t>
+        </is>
+      </c>
+      <c r="J37" s="26" t="inlineStr">
+        <is>
+          <t>Ideia</t>
+        </is>
+      </c>
+      <c r="K37" s="23" t="inlineStr">
+        <is>
+          <t>Vídeo de som ambiente, 30 segundos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="78" customHeight="1" s="16">
+      <c r="A38" s="22" t="n">
+        <v>46366</v>
+      </c>
+      <c r="B38" s="23">
+        <f>TEXT(A38,"dddd")</f>
+        <v/>
+      </c>
+      <c r="C38" s="23" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="D38" s="23" t="inlineStr">
+        <is>
+          <t>Reels</t>
+        </is>
+      </c>
+      <c r="E38" s="23" t="inlineStr">
+        <is>
+          <t>Campanha</t>
+        </is>
+      </c>
+      <c r="F38" s="23" t="inlineStr">
+        <is>
+          <t>Traga um amigo</t>
+        </is>
+      </c>
+      <c r="G38" s="23" t="inlineStr">
+        <is>
+          <t>Traga um amigo para a Vila Mathilde. Vocês dois ganham uma condição especial.</t>
+        </is>
+      </c>
+      <c r="H38" s="23" t="inlineStr">
+        <is>
+          <t>#TragaUmAmigo #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+        </is>
+      </c>
+      <c r="I38" s="23" t="inlineStr">
+        <is>
+          <t>Dono</t>
+        </is>
+      </c>
+      <c r="J38" s="26" t="inlineStr">
+        <is>
+          <t>Ideia</t>
+        </is>
+      </c>
+      <c r="K38" s="23" t="inlineStr">
+        <is>
+          <t>Regra do programa a definir com o dono.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="78" customHeight="1" s="16">
+      <c r="A39" s="22" t="n">
+        <v>46367</v>
+      </c>
+      <c r="B39" s="23">
+        <f>TEXT(A39,"dddd")</f>
+        <v/>
+      </c>
+      <c r="C39" s="23" t="inlineStr">
+        <is>
+          <t>Google Perfil</t>
+        </is>
+      </c>
+      <c r="D39" s="23" t="inlineStr">
+        <is>
+          <t>Post</t>
+        </is>
+      </c>
+      <c r="E39" s="23" t="inlineStr">
+        <is>
+          <t>Experiência</t>
+        </is>
+      </c>
+      <c r="F39" s="23" t="inlineStr">
+        <is>
+          <t>Café da manhã e quarto</t>
+        </is>
+      </c>
+      <c r="G39" s="23" t="inlineStr">
+        <is>
+          <t>Café da roça incluso, quarto silencioso e cama confortável. Venha ver.</t>
+        </is>
+      </c>
+      <c r="H39" s="23" t="inlineStr">
+        <is>
+          <t>#VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+        </is>
+      </c>
+      <c r="I39" s="23" t="inlineStr">
+        <is>
+          <t>Dono</t>
+        </is>
+      </c>
+      <c r="J39" s="26" t="inlineStr">
+        <is>
+          <t>Ideia</t>
+        </is>
+      </c>
+      <c r="K39" s="23" t="inlineStr">
+        <is>
+          <t>Subir fotos novas e responder às avaliações.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="78" customHeight="1" s="16">
+      <c r="A40" s="22" t="n">
+        <v>46368</v>
+      </c>
+      <c r="B40" s="23">
+        <f>TEXT(A40,"dddd")</f>
+        <v/>
+      </c>
+      <c r="C40" s="23" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="D40" s="23" t="inlineStr">
+        <is>
+          <t>Transmissão</t>
+        </is>
+      </c>
+      <c r="E40" s="23" t="inlineStr">
+        <is>
+          <t>Campanha</t>
+        </is>
+      </c>
+      <c r="F40" s="23" t="inlineStr">
+        <is>
+          <t>Bilhete de Volta</t>
+        </is>
+      </c>
+      <c r="G40" s="23" t="inlineStr">
+        <is>
+          <t>Quem já se hospedou tem o Bilhete de Volta, com desconto na segunda estadia. Quer usar o seu?</t>
+        </is>
+      </c>
+      <c r="H40" s="23" t="inlineStr">
+        <is>
+          <t>#VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+        </is>
+      </c>
+      <c r="I40" s="23" t="inlineStr">
+        <is>
+          <t>Dono</t>
+        </is>
+      </c>
+      <c r="J40" s="26" t="inlineStr">
+        <is>
+          <t>Ideia</t>
+        </is>
+      </c>
+      <c r="K40" s="23" t="inlineStr">
+        <is>
+          <t>Enviar à lista de ex-hóspedes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="78" customHeight="1" s="16">
+      <c r="A41" s="22" t="n">
+        <v>46370</v>
+      </c>
+      <c r="B41" s="23">
+        <f>TEXT(A41,"dddd")</f>
+        <v/>
+      </c>
+      <c r="C41" s="23" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="D41" s="23" t="inlineStr">
+        <is>
+          <t>Reels</t>
+        </is>
+      </c>
+      <c r="E41" s="23" t="inlineStr">
+        <is>
+          <t>Destino</t>
+        </is>
+      </c>
+      <c r="F41" s="23" t="inlineStr">
+        <is>
+          <t>O verão das cachoeiras</t>
+        </is>
+      </c>
+      <c r="G41" s="23" t="inlineStr">
+        <is>
+          <t>No verão, Matilde é a temporada das cachoeiras. Venha se refrescar e descansar.</t>
+        </is>
+      </c>
+      <c r="H41" s="23" t="inlineStr">
+        <is>
+          <t>#VeraoNaSerra #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+        </is>
+      </c>
+      <c r="I41" s="23" t="inlineStr">
+        <is>
+          <t>Dono</t>
+        </is>
+      </c>
+      <c r="J41" s="26" t="inlineStr">
+        <is>
+          <t>Ideia</t>
+        </is>
+      </c>
+      <c r="K41" s="23" t="inlineStr">
+        <is>
+          <t>Gravar a cachoeira com plano aberto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="78" customHeight="1" s="16">
+      <c r="A42" s="22" t="n">
+        <v>46371</v>
+      </c>
+      <c r="B42" s="23">
+        <f>TEXT(A42,"dddd")</f>
+        <v/>
+      </c>
+      <c r="C42" s="23" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="D42" s="23" t="inlineStr">
+        <is>
+          <t>Vídeo curto</t>
+        </is>
+      </c>
+      <c r="E42" s="23" t="inlineStr">
+        <is>
+          <t>Bastidores</t>
+        </is>
+      </c>
+      <c r="F42" s="23" t="inlineStr">
+        <is>
+          <t>A pousada se vestindo de Natal</t>
+        </is>
+      </c>
+      <c r="G42" s="23" t="inlineStr">
+        <is>
+          <t>A casa já está ficando pronta para o Natal. Venha passar essas datas com a gente.</t>
+        </is>
+      </c>
+      <c r="H42" s="23" t="inlineStr">
+        <is>
+          <t>#NatalEmMatilde #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+        </is>
+      </c>
+      <c r="I42" s="23" t="inlineStr">
+        <is>
+          <t>Dono</t>
+        </is>
+      </c>
+      <c r="J42" s="26" t="inlineStr">
+        <is>
+          <t>Ideia</t>
+        </is>
+      </c>
+      <c r="K42" s="23" t="inlineStr">
+        <is>
+          <t>Mostrar só a decoração que a pousada já tem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="78" customHeight="1" s="16">
+      <c r="A43" s="22" t="n">
+        <v>46372</v>
+      </c>
+      <c r="B43" s="23">
+        <f>TEXT(A43,"dddd")</f>
+        <v/>
+      </c>
+      <c r="C43" s="23" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="D43" s="23" t="inlineStr">
+        <is>
+          <t>Vídeo</t>
+        </is>
+      </c>
+      <c r="E43" s="23" t="inlineStr">
+        <is>
+          <t>Campanha</t>
+        </is>
+      </c>
+      <c r="F43" s="23" t="inlineStr">
+        <is>
+          <t>Natal em Matilde</t>
+        </is>
+      </c>
+      <c r="G43" s="23" t="inlineStr">
+        <is>
+          <t>Um Natal tranquilo, entre montanhas e cachoeiras. Reserve pelo WhatsApp.</t>
+        </is>
+      </c>
+      <c r="H43" s="23" t="inlineStr">
+        <is>
+          <t>#NatalEmMatilde #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+        </is>
+      </c>
+      <c r="I43" s="23" t="inlineStr">
+        <is>
+          <t>Dono</t>
+        </is>
+      </c>
+      <c r="J43" s="26" t="inlineStr">
+        <is>
+          <t>Ideia</t>
+        </is>
+      </c>
+      <c r="K43" s="23" t="inlineStr">
+        <is>
+          <t>Incluir chamada para o WhatsApp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="78" customHeight="1" s="16">
+      <c r="A44" s="22" t="n">
+        <v>46373</v>
+      </c>
+      <c r="B44" s="23">
+        <f>TEXT(A44,"dddd")</f>
+        <v/>
+      </c>
+      <c r="C44" s="23" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="D44" s="23" t="inlineStr">
+        <is>
+          <t>Reels</t>
+        </is>
+      </c>
+      <c r="E44" s="23" t="inlineStr">
+        <is>
+          <t>Experiência</t>
+        </is>
+      </c>
+      <c r="F44" s="23" t="inlineStr">
+        <is>
+          <t>A piscina no calor</t>
+        </is>
+      </c>
+      <c r="G44" s="23" t="inlineStr">
+        <is>
+          <t>Calor de dezembro pede piscina e sombra. A nossa está esperando por você.</t>
+        </is>
+      </c>
+      <c r="H44" s="23" t="inlineStr">
+        <is>
+          <t>#Sossego #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+        </is>
+      </c>
+      <c r="I44" s="23" t="inlineStr">
+        <is>
+          <t>Dono</t>
+        </is>
+      </c>
+      <c r="J44" s="26" t="inlineStr">
+        <is>
+          <t>Ideia</t>
+        </is>
+      </c>
+      <c r="K44" s="23" t="inlineStr">
+        <is>
+          <t>Gravar sem hóspedes no enquadramento ou com autorização.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="78" customHeight="1" s="16">
+      <c r="A45" s="22" t="n">
+        <v>46374</v>
+      </c>
+      <c r="B45" s="23">
+        <f>TEXT(A45,"dddd")</f>
+        <v/>
+      </c>
+      <c r="C45" s="23" t="inlineStr">
+        <is>
+          <t>Google Perfil</t>
+        </is>
+      </c>
+      <c r="D45" s="23" t="inlineStr">
+        <is>
+          <t>Post</t>
+        </is>
+      </c>
+      <c r="E45" s="23" t="inlineStr">
+        <is>
+          <t>Campanha</t>
+        </is>
+      </c>
+      <c r="F45" s="23" t="inlineStr">
+        <is>
+          <t>Réveillon: poucos quartos</t>
+        </is>
+      </c>
+      <c r="G45" s="23" t="inlineStr">
+        <is>
+          <t>Quer começar o ano em paz? Restam poucos quartos para o Réveillon. Chame no WhatsApp.</t>
+        </is>
+      </c>
+      <c r="H45" s="23" t="inlineStr">
+        <is>
+          <t>#VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+        </is>
+      </c>
+      <c r="I45" s="23" t="inlineStr">
+        <is>
+          <t>Dono</t>
+        </is>
+      </c>
+      <c r="J45" s="26" t="inlineStr">
+        <is>
+          <t>Ideia</t>
+        </is>
+      </c>
+      <c r="K45" s="23" t="inlineStr">
+        <is>
+          <t>Confirmar a disponibilidade antes de publicar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="78" customHeight="1" s="16">
+      <c r="A46" s="22" t="n">
+        <v>46375</v>
+      </c>
+      <c r="B46" s="23">
+        <f>TEXT(A46,"dddd")</f>
+        <v/>
+      </c>
+      <c r="C46" s="23" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="D46" s="23" t="inlineStr">
+        <is>
+          <t>Transmissão</t>
+        </is>
+      </c>
+      <c r="E46" s="23" t="inlineStr">
+        <is>
+          <t>Campanha</t>
+        </is>
+      </c>
+      <c r="F46" s="23" t="inlineStr">
+        <is>
+          <t>Presente de Natal: vale-estadia</t>
+        </is>
+      </c>
+      <c r="G46" s="23" t="inlineStr">
+        <is>
+          <t>Que tal presentear alguém com uma estadia em Matilde? Responda aqui e a gente explica.</t>
+        </is>
+      </c>
+      <c r="H46" s="23" t="inlineStr">
+        <is>
+          <t>#VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+        </is>
+      </c>
+      <c r="I46" s="23" t="inlineStr">
+        <is>
+          <t>Dono</t>
+        </is>
+      </c>
+      <c r="J46" s="26" t="inlineStr">
+        <is>
+          <t>Ideia</t>
+        </is>
+      </c>
+      <c r="K46" s="23" t="inlineStr">
+        <is>
+          <t>Regra do vale-estadia a definir com o dono.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="78" customHeight="1" s="16">
+      <c r="A47" s="22" t="n">
+        <v>46377</v>
+      </c>
+      <c r="B47" s="23">
+        <f>TEXT(A47,"dddd")</f>
+        <v/>
+      </c>
+      <c r="C47" s="23" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="D47" s="23" t="inlineStr">
+        <is>
+          <t>Reels</t>
+        </is>
+      </c>
+      <c r="E47" s="23" t="inlineStr">
+        <is>
+          <t>Depoimento</t>
+        </is>
+      </c>
+      <c r="F47" s="23" t="inlineStr">
+        <is>
+          <t>Obrigado pelo ano</t>
+        </is>
+      </c>
+      <c r="G47" s="23" t="inlineStr">
+        <is>
+          <t>O que mais ouvimos neste ano: atendimento de família e sossego. Obrigado por confiar na gente.</t>
+        </is>
+      </c>
+      <c r="H47" s="23" t="inlineStr">
+        <is>
+          <t>#Depoimento #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+        </is>
+      </c>
+      <c r="I47" s="23" t="inlineStr">
+        <is>
+          <t>Dono</t>
+        </is>
+      </c>
+      <c r="J47" s="26" t="inlineStr">
+        <is>
+          <t>Ideia</t>
+        </is>
+      </c>
+      <c r="K47" s="23" t="inlineStr">
+        <is>
+          <t>Só depoimentos autorizados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="78" customHeight="1" s="16">
+      <c r="A48" s="22" t="n">
+        <v>46378</v>
+      </c>
+      <c r="B48" s="23">
+        <f>TEXT(A48,"dddd")</f>
+        <v/>
+      </c>
+      <c r="C48" s="23" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="D48" s="23" t="inlineStr">
+        <is>
+          <t>Vídeo curto</t>
+        </is>
+      </c>
+      <c r="E48" s="23" t="inlineStr">
+        <is>
+          <t>Experiência</t>
+        </is>
+      </c>
+      <c r="F48" s="23" t="inlineStr">
+        <is>
+          <t>Quarto pronto para as festas</t>
+        </is>
+      </c>
+      <c r="G48" s="23" t="inlineStr">
+        <is>
+          <t>Lençol limpo, rede armada e um bilhete de boas-vindas. É assim que a gente recebe.</t>
+        </is>
+      </c>
+      <c r="H48" s="23" t="inlineStr">
+        <is>
+          <t>#PousadaDeMontanha #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+        </is>
+      </c>
+      <c r="I48" s="23" t="inlineStr">
+        <is>
+          <t>Dono</t>
+        </is>
+      </c>
+      <c r="J48" s="26" t="inlineStr">
+        <is>
+          <t>Ideia</t>
+        </is>
+      </c>
+      <c r="K48" s="23" t="inlineStr">
+        <is>
+          <t>Vídeo de 15 segundos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="78" customHeight="1" s="16">
+      <c r="A49" s="22" t="n">
+        <v>46379</v>
+      </c>
+      <c r="B49" s="23">
+        <f>TEXT(A49,"dddd")</f>
+        <v/>
+      </c>
+      <c r="C49" s="23" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="D49" s="23" t="inlineStr">
+        <is>
+          <t>Vídeo</t>
+        </is>
+      </c>
+      <c r="E49" s="23" t="inlineStr">
+        <is>
+          <t>Campanha</t>
+        </is>
+      </c>
+      <c r="F49" s="23" t="inlineStr">
+        <is>
+          <t>Última chamada do Natal</t>
+        </is>
+      </c>
+      <c r="G49" s="23" t="inlineStr">
+        <is>
+          <t>Ainda dá tempo de passar o Natal em Matilde. Chame no WhatsApp.</t>
+        </is>
+      </c>
+      <c r="H49" s="23" t="inlineStr">
+        <is>
+          <t>#NatalEmMatilde #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+        </is>
+      </c>
+      <c r="I49" s="23" t="inlineStr">
+        <is>
+          <t>Dono</t>
+        </is>
+      </c>
+      <c r="J49" s="26" t="inlineStr">
+        <is>
+          <t>Ideia</t>
+        </is>
+      </c>
+      <c r="K49" s="23" t="inlineStr">
+        <is>
+          <t>Publicar só se houver quartos livres.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="78" customHeight="1" s="16">
+      <c r="A50" s="22" t="n">
+        <v>46380</v>
+      </c>
+      <c r="B50" s="23">
+        <f>TEXT(A50,"dddd")</f>
+        <v/>
+      </c>
+      <c r="C50" s="23" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="D50" s="23" t="inlineStr">
+        <is>
+          <t>Reels</t>
+        </is>
+      </c>
+      <c r="E50" s="23" t="inlineStr">
+        <is>
+          <t>Bastidores</t>
+        </is>
+      </c>
+      <c r="F50" s="23" t="inlineStr">
+        <is>
+          <t>Feliz Natal dos anfitriões</t>
+        </is>
+      </c>
+      <c r="G50" s="23" t="inlineStr">
+        <is>
+          <t>Desejamos um Natal de paz para você e sua família. Com carinho, a família da Vila Mathilde.</t>
+        </is>
+      </c>
+      <c r="H50" s="23" t="inlineStr">
+        <is>
+          <t>#FelizNatal #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+        </is>
+      </c>
+      <c r="I50" s="23" t="inlineStr">
+        <is>
+          <t>Dono</t>
+        </is>
+      </c>
+      <c r="J50" s="26" t="inlineStr">
+        <is>
+          <t>Ideia</t>
+        </is>
+      </c>
+      <c r="K50" s="23" t="inlineStr">
+        <is>
+          <t>Vídeo curto com os anfitriões, com autorização.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="78" customHeight="1" s="16">
+      <c r="A51" s="22" t="n">
+        <v>46382</v>
+      </c>
+      <c r="B51" s="23">
+        <f>TEXT(A51,"dddd")</f>
+        <v/>
+      </c>
+      <c r="C51" s="23" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="D51" s="23" t="inlineStr">
+        <is>
+          <t>Transmissão</t>
+        </is>
+      </c>
+      <c r="E51" s="23" t="inlineStr">
+        <is>
+          <t>Campanha</t>
+        </is>
+      </c>
+      <c r="F51" s="23" t="inlineStr">
+        <is>
+          <t>Réveillon e verão: datas livres</t>
+        </is>
+      </c>
+      <c r="G51" s="23" t="inlineStr">
+        <is>
+          <t>Se você quer começar 2027 com sossego, ainda temos algumas datas. Responda aqui.</t>
+        </is>
+      </c>
+      <c r="H51" s="23" t="inlineStr">
+        <is>
+          <t>#VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+        </is>
+      </c>
+      <c r="I51" s="23" t="inlineStr">
+        <is>
+          <t>Dono</t>
+        </is>
+      </c>
+      <c r="J51" s="26" t="inlineStr">
+        <is>
+          <t>Ideia</t>
+        </is>
+      </c>
+      <c r="K51" s="23" t="inlineStr">
+        <is>
+          <t>Conferir a disponibilidade.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="78" customHeight="1" s="16">
+      <c r="A52" s="28" t="n">
+        <v>46384</v>
+      </c>
+      <c r="B52" s="29">
+        <f>TEXT(A52,"dddd")</f>
+        <v/>
+      </c>
+      <c r="C52" s="29" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="D52" s="29" t="inlineStr">
+        <is>
+          <t>Reels</t>
+        </is>
+      </c>
+      <c r="E52" s="29" t="inlineStr">
+        <is>
+          <t>Destino</t>
+        </is>
+      </c>
+      <c r="F52" s="29" t="inlineStr">
+        <is>
+          <t>Fim de ano na cachoeira</t>
+        </is>
+      </c>
+      <c r="G52" s="29" t="inlineStr">
+        <is>
+          <t>Fim de ano com cachoeira, estação e muito descanso. Venha para Matilde.</t>
+        </is>
+      </c>
+      <c r="H52" s="29" t="inlineStr">
+        <is>
+          <t>#FimDeAno #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+        </is>
+      </c>
+      <c r="I52" s="29" t="inlineStr">
+        <is>
+          <t>Dono</t>
+        </is>
+      </c>
+      <c r="J52" s="30" t="inlineStr">
+        <is>
+          <t>Ideia</t>
+        </is>
+      </c>
+      <c r="K52" s="29" t="inlineStr">
+        <is>
+          <t>Reaproveitar imagens do mês.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="78" customHeight="1" s="16">
+      <c r="A53" s="28" t="n">
+        <v>46385</v>
+      </c>
+      <c r="B53" s="29">
+        <f>TEXT(A53,"dddd")</f>
+        <v/>
+      </c>
+      <c r="C53" s="29" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="D53" s="29" t="inlineStr">
+        <is>
+          <t>Vídeo curto</t>
+        </is>
+      </c>
+      <c r="E53" s="29" t="inlineStr">
+        <is>
+          <t>Campanha</t>
+        </is>
+      </c>
+      <c r="F53" s="29" t="inlineStr">
+        <is>
+          <t>Bilhete de Volta para 2027</t>
+        </is>
+      </c>
+      <c r="G53" s="29" t="inlineStr">
+        <is>
+          <t>Quem se hospeda agora leva o Bilhete de Volta para usar em 2027.</t>
+        </is>
+      </c>
+      <c r="H53" s="29" t="inlineStr">
+        <is>
+          <t>#BilheteDeVolta #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+        </is>
+      </c>
+      <c r="I53" s="29" t="inlineStr">
+        <is>
+          <t>Dono</t>
+        </is>
+      </c>
+      <c r="J53" s="30" t="inlineStr">
+        <is>
+          <t>Ideia</t>
+        </is>
+      </c>
+      <c r="K53" s="29" t="inlineStr">
+        <is>
+          <t>Regra do desconto a definir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="78" customHeight="1" s="16">
+      <c r="A54" s="28" t="n">
+        <v>46386</v>
+      </c>
+      <c r="B54" s="29">
+        <f>TEXT(A54,"dddd")</f>
+        <v/>
+      </c>
+      <c r="C54" s="29" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="D54" s="29" t="inlineStr">
+        <is>
+          <t>Vídeo</t>
+        </is>
+      </c>
+      <c r="E54" s="29" t="inlineStr">
+        <is>
+          <t>Depoimento</t>
+        </is>
+      </c>
+      <c r="F54" s="29" t="inlineStr">
+        <is>
+          <t>Obrigado, 2026</t>
+        </is>
+      </c>
+      <c r="G54" s="29" t="inlineStr">
+        <is>
+          <t>Obrigado a todos que passaram por aqui em 2026. Até o próximo ano.</t>
+        </is>
+      </c>
+      <c r="H54" s="29" t="inlineStr">
+        <is>
+          <t>#Obrigado #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+        </is>
+      </c>
+      <c r="I54" s="29" t="inlineStr">
+        <is>
+          <t>Dono</t>
+        </is>
+      </c>
+      <c r="J54" s="30" t="inlineStr">
+        <is>
+          <t>Ideia</t>
+        </is>
+      </c>
+      <c r="K54" s="29" t="inlineStr">
+        <is>
+          <t>Montagem curta com os melhores momentos autorizados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="78" customHeight="1" s="16">
+      <c r="A55" s="28" t="n">
+        <v>46387</v>
+      </c>
+      <c r="B55" s="29">
+        <f>TEXT(A55,"dddd")</f>
+        <v/>
+      </c>
+      <c r="C55" s="29" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="D55" s="29" t="inlineStr">
+        <is>
+          <t>Reels</t>
+        </is>
+      </c>
+      <c r="E55" s="29" t="inlineStr">
+        <is>
+          <t>Campanha</t>
+        </is>
+      </c>
+      <c r="F55" s="29" t="inlineStr">
+        <is>
+          <t>Boas festas e feliz 2027</t>
+        </is>
+      </c>
+      <c r="G55" s="29" t="inlineStr">
+        <is>
+          <t>Que 2027 comece com sossego. Feliz Ano Novo de toda a Vila Mathilde.</t>
+        </is>
+      </c>
+      <c r="H55" s="29" t="inlineStr">
+        <is>
+          <t>#FelizAnoNovo #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+        </is>
+      </c>
+      <c r="I55" s="29" t="inlineStr">
+        <is>
+          <t>Dono</t>
+        </is>
+      </c>
+      <c r="J55" s="30" t="inlineStr">
+        <is>
+          <t>Ideia</t>
+        </is>
+      </c>
+      <c r="K55" s="29" t="inlineStr">
+        <is>
+          <t>Vídeo de encerramento do ano.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:K2"/>

</xml_diff>

<commit_message>
Calendario com dias variados e sempre com conteudo no fim de semana
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/08-calendario-estrategico.xlsx
+++ b/08-calendario-estrategico.xlsx
@@ -751,7 +751,7 @@
     <row r="2" ht="15" customHeight="1" s="16">
       <c r="A2" s="15" t="inlineStr">
         <is>
-          <t>Pousada Vila Mathilde: novembro e dezembro de 2026. Três publicações por semana, em dias alternados (segunda, quarta e sexta), com conteúdo útil para quem decide a viagem.</t>
+          <t>Pousada Vila Mathilde: novembro e dezembro de 2026. Publicações em dias variados da semana, sem ritmo fixo, e sempre com conteúdo no sábado ou no domingo (26 publicações).</t>
         </is>
       </c>
     </row>
@@ -814,7 +814,7 @@
     </row>
     <row r="5" ht="78" customHeight="1" s="16">
       <c r="A5" s="22" t="n">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="B5" s="23">
         <f>TEXT(A5,"dddd")</f>
@@ -868,7 +868,7 @@
     </row>
     <row r="6" ht="78" customHeight="1" s="16">
       <c r="A6" s="22" t="n">
-        <v>46330</v>
+        <v>46331</v>
       </c>
       <c r="B6" s="23">
         <f>TEXT(A6,"dddd")</f>
@@ -909,9 +909,9 @@
           <t>Dono</t>
         </is>
       </c>
-      <c r="J6" s="24" t="inlineStr">
-        <is>
-          <t>Em produção</t>
+      <c r="J6" s="26" t="inlineStr">
+        <is>
+          <t>Ideia</t>
         </is>
       </c>
       <c r="K6" s="23" t="inlineStr">
@@ -922,7 +922,7 @@
     </row>
     <row r="7" ht="78" customHeight="1" s="16">
       <c r="A7" s="22" t="n">
-        <v>46332</v>
+        <v>46333</v>
       </c>
       <c r="B7" s="23">
         <f>TEXT(A7,"dddd")</f>
@@ -930,32 +930,32 @@
       </c>
       <c r="C7" s="25" t="inlineStr">
         <is>
-          <t>Google Perfil</t>
+          <t>Instagram</t>
         </is>
       </c>
       <c r="D7" s="25" t="inlineStr">
         <is>
-          <t>Post</t>
+          <t>Reels</t>
         </is>
       </c>
       <c r="E7" s="25" t="inlineStr">
         <is>
-          <t>Campanha</t>
+          <t>Destino</t>
         </is>
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>Sossego de Meio de Semana</t>
+          <t>O túnel de Matilde, pelos trilhos</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>De domingo a quinta a pousada é só sossego. Pergunte pelo pacote do meio da semana. Chame no WhatsApp pelo botão do perfil.</t>
+          <t>Da estação até o túnel, o caminho é pelos trilhos. Água na altura do tornozelo e uma pedra que guarda história. Leve lanterna e calçado adequado.</t>
         </is>
       </c>
       <c r="H7" s="25" t="inlineStr">
         <is>
-          <t>#VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+          <t>#TunelDeMatilde #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
         </is>
       </c>
       <c r="I7" s="23" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="K7" s="25" t="inlineStr">
         <is>
-          <t>Preço do pacote a definir com o dono. Incluir foto real do quarto.</t>
+          <t>Orientação de segurança do diagnóstico: lanterna e calçado adequado.</t>
         </is>
       </c>
     </row>
@@ -984,32 +984,32 @@
       </c>
       <c r="C8" s="23" t="inlineStr">
         <is>
-          <t>Instagram</t>
+          <t>TikTok</t>
         </is>
       </c>
       <c r="D8" s="23" t="inlineStr">
         <is>
-          <t>Reels</t>
+          <t>Vídeo curto</t>
         </is>
       </c>
       <c r="E8" s="23" t="inlineStr">
         <is>
-          <t>Destino</t>
+          <t>Experiência</t>
         </is>
       </c>
       <c r="F8" s="23" t="inlineStr">
         <is>
-          <t>O túnel de Matilde, pelos trilhos</t>
+          <t>O que está incluso na diária</t>
         </is>
       </c>
       <c r="G8" s="23" t="inlineStr">
         <is>
-          <t>Da estação até o túnel, o caminho é pelos trilhos. Água na altura do tornozelo e uma pedra que guarda história. Leve lanterna e calçado adequado.</t>
+          <t>Café da manhã da roça, estacionamento, piscina e área para petiscos. Veja o que você leva quando reserva na Vila Mathilde.</t>
         </is>
       </c>
       <c r="H8" s="23" t="inlineStr">
         <is>
-          <t>#TunelDeMatilde #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+          <t>#Diaria #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
         </is>
       </c>
       <c r="I8" s="23" t="inlineStr">
@@ -1024,7 +1024,7 @@
       </c>
       <c r="K8" s="23" t="inlineStr">
         <is>
-          <t>Orientação de segurança do diagnóstico: lanterna e calçado adequado.</t>
+          <t>Confirmar a lista de itens com o dono antes de gravar.</t>
         </is>
       </c>
     </row>
@@ -1038,32 +1038,32 @@
       </c>
       <c r="C9" s="23" t="inlineStr">
         <is>
-          <t>TikTok</t>
+          <t>Google Perfil</t>
         </is>
       </c>
       <c r="D9" s="23" t="inlineStr">
         <is>
-          <t>Vídeo curto</t>
+          <t>Post</t>
         </is>
       </c>
       <c r="E9" s="23" t="inlineStr">
         <is>
-          <t>Experiência</t>
+          <t>Campanha</t>
         </is>
       </c>
       <c r="F9" s="23" t="inlineStr">
         <is>
-          <t>O que está incluso na diária</t>
+          <t>Sossego de Meio de Semana</t>
         </is>
       </c>
       <c r="G9" s="23" t="inlineStr">
         <is>
-          <t>Café da manhã da roça, estacionamento, piscina e área para petiscos. Veja o que você leva quando reserva na Vila Mathilde.</t>
+          <t>De domingo a quinta a pousada é só sossego. Pergunte pelo pacote do meio da semana. Chame no WhatsApp pelo botão do perfil.</t>
         </is>
       </c>
       <c r="H9" s="23" t="inlineStr">
         <is>
-          <t>#Diaria #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+          <t>#VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
         </is>
       </c>
       <c r="I9" s="23" t="inlineStr">
@@ -1078,13 +1078,13 @@
       </c>
       <c r="K9" s="23" t="inlineStr">
         <is>
-          <t>Confirmar a lista de itens com o dono antes de gravar.</t>
+          <t>Preço do pacote a definir com o dono. Incluir foto real do quarto.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="78" customHeight="1" s="16">
       <c r="A10" s="22" t="n">
-        <v>46339</v>
+        <v>46341</v>
       </c>
       <c r="B10" s="23">
         <f>TEXT(A10,"dddd")</f>
@@ -1092,12 +1092,12 @@
       </c>
       <c r="C10" s="23" t="inlineStr">
         <is>
-          <t>WhatsApp</t>
+          <t>Instagram</t>
         </is>
       </c>
       <c r="D10" s="23" t="inlineStr">
         <is>
-          <t>Transmissão</t>
+          <t>Reels</t>
         </is>
       </c>
       <c r="E10" s="23" t="inlineStr">
@@ -1107,17 +1107,17 @@
       </c>
       <c r="F10" s="23" t="inlineStr">
         <is>
-          <t>Visitante de excursão: volte e durma</t>
+          <t>Bilhete de Volta</t>
         </is>
       </c>
       <c r="G10" s="23" t="inlineStr">
         <is>
-          <t>Esteve em Matilde de excursão? Volte e durma na Vila Mathilde, com condição especial para quem já conhece a cachoeira. Responda aqui.</t>
+          <t>Gostou da estadia? Leve o Bilhete de Volta: um desconto na sua segunda vez em Matilde.</t>
         </is>
       </c>
       <c r="H10" s="23" t="inlineStr">
         <is>
-          <t>#VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+          <t>#BilheteDeVolta #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
         </is>
       </c>
       <c r="I10" s="23" t="inlineStr">
@@ -1132,13 +1132,13 @@
       </c>
       <c r="K10" s="23" t="inlineStr">
         <is>
-          <t>Enviar à lista formada pelo QR code do centrinho, da estação e da cachoeira.</t>
+          <t>Regra do desconto a definir com o dono.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="78" customHeight="1" s="16">
       <c r="A11" s="22" t="n">
-        <v>46342</v>
+        <v>46343</v>
       </c>
       <c r="B11" s="23">
         <f>TEXT(A11,"dddd")</f>
@@ -1156,22 +1156,22 @@
       </c>
       <c r="E11" s="23" t="inlineStr">
         <is>
-          <t>Campanha</t>
+          <t>Experiência</t>
         </is>
       </c>
       <c r="F11" s="23" t="inlineStr">
         <is>
-          <t>Bilhete de Volta</t>
+          <t>As perguntas que mais recebemos</t>
         </is>
       </c>
       <c r="G11" s="23" t="inlineStr">
         <is>
-          <t>Gostou da estadia? Leve o Bilhete de Volta: um desconto na sua segunda vez em Matilde.</t>
+          <t>Tem café da manhã? Tem. Aceita pets? Não aceitamos. Crianças? Cobramos à parte. Qualquer outra dúvida, chame no WhatsApp.</t>
         </is>
       </c>
       <c r="H11" s="23" t="inlineStr">
         <is>
-          <t>#BilheteDeVolta #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+          <t>#Duvidas #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
         </is>
       </c>
       <c r="I11" s="23" t="inlineStr">
@@ -1186,13 +1186,13 @@
       </c>
       <c r="K11" s="23" t="inlineStr">
         <is>
-          <t>Regra do desconto a definir com o dono.</t>
+          <t>Confirmar as políticas atuais da pousada com o dono. Evitar surpresa na hora da reserva.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="78" customHeight="1" s="16">
       <c r="A12" s="22" t="n">
-        <v>46344</v>
+        <v>46345</v>
       </c>
       <c r="B12" s="23">
         <f>TEXT(A12,"dddd")</f>
@@ -1246,7 +1246,7 @@
     </row>
     <row r="13" ht="78" customHeight="1" s="16">
       <c r="A13" s="22" t="n">
-        <v>46346</v>
+        <v>46347</v>
       </c>
       <c r="B13" s="23">
         <f>TEXT(A13,"dddd")</f>
@@ -1354,7 +1354,7 @@
     </row>
     <row r="15" ht="78" customHeight="1" s="16">
       <c r="A15" s="22" t="n">
-        <v>46351</v>
+        <v>46353</v>
       </c>
       <c r="B15" s="23">
         <f>TEXT(A15,"dddd")</f>
@@ -1362,12 +1362,12 @@
       </c>
       <c r="C15" s="23" t="inlineStr">
         <is>
-          <t>Instagram</t>
+          <t>WhatsApp</t>
         </is>
       </c>
       <c r="D15" s="23" t="inlineStr">
         <is>
-          <t>Reels</t>
+          <t>Transmissão</t>
         </is>
       </c>
       <c r="E15" s="23" t="inlineStr">
@@ -1377,22 +1377,22 @@
       </c>
       <c r="F15" s="23" t="inlineStr">
         <is>
-          <t>Roteiro de 2 dias com criador</t>
+          <t>Visitante de excursão: volte e durma</t>
         </is>
       </c>
       <c r="G15" s="23" t="inlineStr">
         <is>
-          <t>Primeiro dia: cachoeira e mirante. Segundo dia: estação e túnel. No meio, o descanso na Vila Mathilde.</t>
+          <t>Esteve em Matilde de excursão? Volte e durma na Vila Mathilde, com condição especial para quem já conhece a cachoeira. Responda aqui.</t>
         </is>
       </c>
       <c r="H15" s="23" t="inlineStr">
         <is>
-          <t>#RoteiroDe2Dias #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+          <t>#VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
         </is>
       </c>
       <c r="I15" s="23" t="inlineStr">
         <is>
-          <t>Criador parceiro</t>
+          <t>Dono</t>
         </is>
       </c>
       <c r="J15" s="26" t="inlineStr">
@@ -1402,13 +1402,13 @@
       </c>
       <c r="K15" s="23" t="inlineStr">
         <is>
-          <t>Parceria paga. Briefing e direitos de uso das imagens combinados antes.</t>
+          <t>Enviar à lista formada pelo QR code do centrinho, da estação e da cachoeira.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="78" customHeight="1" s="16">
       <c r="A16" s="22" t="n">
-        <v>46353</v>
+        <v>46355</v>
       </c>
       <c r="B16" s="23">
         <f>TEXT(A16,"dddd")</f>
@@ -1416,37 +1416,37 @@
       </c>
       <c r="C16" s="23" t="inlineStr">
         <is>
-          <t>Google Perfil</t>
+          <t>Instagram</t>
         </is>
       </c>
       <c r="D16" s="23" t="inlineStr">
         <is>
-          <t>Post</t>
+          <t>Reels</t>
         </is>
       </c>
       <c r="E16" s="23" t="inlineStr">
         <is>
-          <t>Depoimento</t>
+          <t>Campanha</t>
         </is>
       </c>
       <c r="F16" s="23" t="inlineStr">
         <is>
-          <t>Obrigado pelas avaliações</t>
+          <t>Roteiro de 2 dias com criador</t>
         </is>
       </c>
       <c r="G16" s="23" t="inlineStr">
         <is>
-          <t>Nota 4,7 no Google. Obrigado a quem já se hospedou com a gente. A sua avaliação ajuda outras pessoas a nos encontrar.</t>
+          <t>Primeiro dia: cachoeira e mirante. Segundo dia: estação e túnel. No meio, o descanso na Vila Mathilde.</t>
         </is>
       </c>
       <c r="H16" s="23" t="inlineStr">
         <is>
-          <t>#VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+          <t>#RoteiroDe2Dias #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
         </is>
       </c>
       <c r="I16" s="23" t="inlineStr">
         <is>
-          <t>Dono</t>
+          <t>Criador parceiro</t>
         </is>
       </c>
       <c r="J16" s="26" t="inlineStr">
@@ -1456,13 +1456,13 @@
       </c>
       <c r="K16" s="23" t="inlineStr">
         <is>
-          <t>Responder também às avaliações recentes.</t>
+          <t>Parceria paga. Briefing e direitos de uso das imagens combinados antes.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="78" customHeight="1" s="16">
       <c r="A17" s="22" t="n">
-        <v>46356</v>
+        <v>46357</v>
       </c>
       <c r="B17" s="23">
         <f>TEXT(A17,"dddd")</f>
@@ -1470,32 +1470,32 @@
       </c>
       <c r="C17" s="23" t="inlineStr">
         <is>
-          <t>Instagram</t>
+          <t>Facebook</t>
         </is>
       </c>
       <c r="D17" s="23" t="inlineStr">
         <is>
-          <t>Reels</t>
+          <t>Vídeo</t>
         </is>
       </c>
       <c r="E17" s="23" t="inlineStr">
         <is>
-          <t>Experiência</t>
+          <t>História</t>
         </is>
       </c>
       <c r="F17" s="23" t="inlineStr">
         <is>
-          <t>As perguntas que mais recebemos</t>
+          <t>Matilde nasceu do trem</t>
         </is>
       </c>
       <c r="G17" s="23" t="inlineStr">
         <is>
-          <t>Tem café da manhã? Tem. Aceita pets? Não aceitamos. Crianças? Cobramos à parte. Qualquer outra dúvida, chame no WhatsApp.</t>
+          <t>O nome Mathilde vem da esposa do engenheiro da ferrovia, segundo relatos locais. Venha conhecer a estação de 1910, tombada pelo Estado.</t>
         </is>
       </c>
       <c r="H17" s="23" t="inlineStr">
         <is>
-          <t>#Duvidas #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+          <t>#EstacaoDeMatilde #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
         </is>
       </c>
       <c r="I17" s="23" t="inlineStr">
@@ -1510,13 +1510,13 @@
       </c>
       <c r="K17" s="23" t="inlineStr">
         <is>
-          <t>Confirmar as políticas atuais da pousada com o dono. Evitar surpresa na hora da reserva.</t>
+          <t>Tratar o nome como relato local. Dados da estação: iPatrimônio, via diagnóstico.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="78" customHeight="1" s="16">
       <c r="A18" s="22" t="n">
-        <v>46358</v>
+        <v>46360</v>
       </c>
       <c r="B18" s="23">
         <f>TEXT(A18,"dddd")</f>
@@ -1524,32 +1524,32 @@
       </c>
       <c r="C18" s="23" t="inlineStr">
         <is>
-          <t>Facebook</t>
+          <t>Google Perfil</t>
         </is>
       </c>
       <c r="D18" s="23" t="inlineStr">
         <is>
-          <t>Vídeo</t>
+          <t>Post</t>
         </is>
       </c>
       <c r="E18" s="23" t="inlineStr">
         <is>
-          <t>História</t>
+          <t>Campanha</t>
         </is>
       </c>
       <c r="F18" s="23" t="inlineStr">
         <is>
-          <t>Matilde nasceu do trem</t>
+          <t>Natal e Réveillon: datas</t>
         </is>
       </c>
       <c r="G18" s="23" t="inlineStr">
         <is>
-          <t>O nome Mathilde vem da esposa do engenheiro da ferrovia, segundo relatos locais. Venha conhecer a estação de 1910, tombada pelo Estado.</t>
+          <t>As datas de fim de ano costumam esgotar. Pergunte pelos quartos livres no WhatsApp.</t>
         </is>
       </c>
       <c r="H18" s="23" t="inlineStr">
         <is>
-          <t>#EstacaoDeMatilde #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+          <t>#VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
         </is>
       </c>
       <c r="I18" s="23" t="inlineStr">
@@ -1564,13 +1564,13 @@
       </c>
       <c r="K18" s="23" t="inlineStr">
         <is>
-          <t>Tratar o nome como relato local. Dados da estação: iPatrimônio, via diagnóstico.</t>
+          <t>Escassez honesta: são só 6 quartos.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="78" customHeight="1" s="16">
       <c r="A19" s="22" t="n">
-        <v>46360</v>
+        <v>46361</v>
       </c>
       <c r="B19" s="23">
         <f>TEXT(A19,"dddd")</f>
@@ -1578,32 +1578,32 @@
       </c>
       <c r="C19" s="23" t="inlineStr">
         <is>
-          <t>Google Perfil</t>
+          <t>Instagram</t>
         </is>
       </c>
       <c r="D19" s="23" t="inlineStr">
         <is>
-          <t>Post</t>
+          <t>Reels</t>
         </is>
       </c>
       <c r="E19" s="23" t="inlineStr">
         <is>
-          <t>Campanha</t>
+          <t>Depoimento</t>
         </is>
       </c>
       <c r="F19" s="23" t="inlineStr">
         <is>
-          <t>Natal e Réveillon: datas</t>
+          <t>Hóspedes que voltaram</t>
         </is>
       </c>
       <c r="G19" s="23" t="inlineStr">
         <is>
-          <t>As datas de fim de ano costumam esgotar. Pergunte pelos quartos livres no WhatsApp.</t>
+          <t>Tem gente que já voltou duas vezes. Obrigado pela confiança, a casa é de vocês.</t>
         </is>
       </c>
       <c r="H19" s="23" t="inlineStr">
         <is>
-          <t>#VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+          <t>#Depoimento #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
         </is>
       </c>
       <c r="I19" s="23" t="inlineStr">
@@ -1618,7 +1618,7 @@
       </c>
       <c r="K19" s="23" t="inlineStr">
         <is>
-          <t>Escassez honesta: são só 6 quartos.</t>
+          <t>Só com autorização de quem aparece.</t>
         </is>
       </c>
     </row>
@@ -1632,32 +1632,32 @@
       </c>
       <c r="C20" s="23" t="inlineStr">
         <is>
-          <t>Instagram</t>
+          <t>TikTok</t>
         </is>
       </c>
       <c r="D20" s="23" t="inlineStr">
         <is>
-          <t>Reels</t>
+          <t>Vídeo curto</t>
         </is>
       </c>
       <c r="E20" s="23" t="inlineStr">
         <is>
-          <t>Depoimento</t>
+          <t>Destino</t>
         </is>
       </c>
       <c r="F20" s="23" t="inlineStr">
         <is>
-          <t>Hóspedes que voltaram</t>
+          <t>A cachoeira cheia depois da chuva</t>
         </is>
       </c>
       <c r="G20" s="23" t="inlineStr">
         <is>
-          <t>Tem gente que já voltou duas vezes. Obrigado pela confiança, a casa é de vocês.</t>
+          <t>Depois da chuva, a cachoeira de Matilde fica ainda mais forte. Vale a espera.</t>
         </is>
       </c>
       <c r="H20" s="23" t="inlineStr">
         <is>
-          <t>#Depoimento #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+          <t>#CachoeiraDeMatilde #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
         </is>
       </c>
       <c r="I20" s="23" t="inlineStr">
@@ -1672,13 +1672,13 @@
       </c>
       <c r="K20" s="23" t="inlineStr">
         <is>
-          <t>Só com autorização de quem aparece.</t>
+          <t>Gravar no dia seguinte à chuva, com cuidado nas escadas.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="78" customHeight="1" s="16">
       <c r="A21" s="22" t="n">
-        <v>46365</v>
+        <v>46366</v>
       </c>
       <c r="B21" s="23">
         <f>TEXT(A21,"dddd")</f>
@@ -1686,32 +1686,32 @@
       </c>
       <c r="C21" s="23" t="inlineStr">
         <is>
-          <t>TikTok</t>
+          <t>WhatsApp</t>
         </is>
       </c>
       <c r="D21" s="23" t="inlineStr">
         <is>
-          <t>Vídeo curto</t>
+          <t>Transmissão</t>
         </is>
       </c>
       <c r="E21" s="23" t="inlineStr">
         <is>
-          <t>Destino</t>
+          <t>Campanha</t>
         </is>
       </c>
       <c r="F21" s="23" t="inlineStr">
         <is>
-          <t>A cachoeira cheia depois da chuva</t>
+          <t>Aniversariantes de dezembro</t>
         </is>
       </c>
       <c r="G21" s="23" t="inlineStr">
         <is>
-          <t>Depois da chuva, a cachoeira de Matilde fica ainda mais forte. Vale a espera.</t>
+          <t>Se o seu aniversário é em dezembro, a gente quer comemorar com você. Responda aqui para saber a condição especial.</t>
         </is>
       </c>
       <c r="H21" s="23" t="inlineStr">
         <is>
-          <t>#CachoeiraDeMatilde #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+          <t>#VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
         </is>
       </c>
       <c r="I21" s="23" t="inlineStr">
@@ -1726,13 +1726,13 @@
       </c>
       <c r="K21" s="23" t="inlineStr">
         <is>
-          <t>Gravar no dia seguinte à chuva, com cuidado nas escadas.</t>
+          <t>Usar só a lista de quem informou a data de aniversário.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="78" customHeight="1" s="16">
       <c r="A22" s="22" t="n">
-        <v>46367</v>
+        <v>46369</v>
       </c>
       <c r="B22" s="23">
         <f>TEXT(A22,"dddd")</f>
@@ -1740,12 +1740,12 @@
       </c>
       <c r="C22" s="23" t="inlineStr">
         <is>
-          <t>WhatsApp</t>
+          <t>Instagram</t>
         </is>
       </c>
       <c r="D22" s="23" t="inlineStr">
         <is>
-          <t>Transmissão</t>
+          <t>Reels</t>
         </is>
       </c>
       <c r="E22" s="23" t="inlineStr">
@@ -1755,17 +1755,17 @@
       </c>
       <c r="F22" s="23" t="inlineStr">
         <is>
-          <t>Aniversariantes de dezembro</t>
+          <t>Traga um amigo</t>
         </is>
       </c>
       <c r="G22" s="23" t="inlineStr">
         <is>
-          <t>Se o seu aniversário é em dezembro, a gente quer comemorar com você. Responda aqui para saber a condição especial.</t>
+          <t>Traga um amigo para a Vila Mathilde. Vocês dois ganham uma condição especial.</t>
         </is>
       </c>
       <c r="H22" s="23" t="inlineStr">
         <is>
-          <t>#VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+          <t>#TragaUmAmigo #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
         </is>
       </c>
       <c r="I22" s="23" t="inlineStr">
@@ -1780,13 +1780,13 @@
       </c>
       <c r="K22" s="23" t="inlineStr">
         <is>
-          <t>Usar só a lista de quem informou a data de aniversário.</t>
+          <t>Regra do programa a definir com o dono.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="78" customHeight="1" s="16">
       <c r="A23" s="22" t="n">
-        <v>46370</v>
+        <v>46372</v>
       </c>
       <c r="B23" s="23">
         <f>TEXT(A23,"dddd")</f>
@@ -1794,12 +1794,12 @@
       </c>
       <c r="C23" s="23" t="inlineStr">
         <is>
-          <t>Instagram</t>
+          <t>Facebook</t>
         </is>
       </c>
       <c r="D23" s="23" t="inlineStr">
         <is>
-          <t>Reels</t>
+          <t>Vídeo</t>
         </is>
       </c>
       <c r="E23" s="23" t="inlineStr">
@@ -1809,17 +1809,17 @@
       </c>
       <c r="F23" s="23" t="inlineStr">
         <is>
-          <t>Traga um amigo</t>
+          <t>Natal em Matilde</t>
         </is>
       </c>
       <c r="G23" s="23" t="inlineStr">
         <is>
-          <t>Traga um amigo para a Vila Mathilde. Vocês dois ganham uma condição especial.</t>
+          <t>Um Natal tranquilo, entre montanhas e cachoeiras. Reserve pelo WhatsApp.</t>
         </is>
       </c>
       <c r="H23" s="23" t="inlineStr">
         <is>
-          <t>#TragaUmAmigo #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+          <t>#NatalEmMatilde #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
         </is>
       </c>
       <c r="I23" s="23" t="inlineStr">
@@ -1834,13 +1834,13 @@
       </c>
       <c r="K23" s="23" t="inlineStr">
         <is>
-          <t>Regra do programa a definir com o dono.</t>
+          <t>Incluir chamada para o WhatsApp.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="78" customHeight="1" s="16">
       <c r="A24" s="22" t="n">
-        <v>46372</v>
+        <v>46373</v>
       </c>
       <c r="B24" s="23">
         <f>TEXT(A24,"dddd")</f>
@@ -1848,12 +1848,12 @@
       </c>
       <c r="C24" s="23" t="inlineStr">
         <is>
-          <t>Facebook</t>
+          <t>Google Perfil</t>
         </is>
       </c>
       <c r="D24" s="23" t="inlineStr">
         <is>
-          <t>Vídeo</t>
+          <t>Post</t>
         </is>
       </c>
       <c r="E24" s="23" t="inlineStr">
@@ -1863,17 +1863,17 @@
       </c>
       <c r="F24" s="23" t="inlineStr">
         <is>
-          <t>Natal em Matilde</t>
+          <t>Réveillon: poucos quartos</t>
         </is>
       </c>
       <c r="G24" s="23" t="inlineStr">
         <is>
-          <t>Um Natal tranquilo, entre montanhas e cachoeiras. Reserve pelo WhatsApp.</t>
+          <t>Quer começar o ano em paz? Restam poucos quartos para o Réveillon. Chame no WhatsApp.</t>
         </is>
       </c>
       <c r="H24" s="23" t="inlineStr">
         <is>
-          <t>#NatalEmMatilde #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+          <t>#VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
         </is>
       </c>
       <c r="I24" s="23" t="inlineStr">
@@ -1888,13 +1888,13 @@
       </c>
       <c r="K24" s="23" t="inlineStr">
         <is>
-          <t>Incluir chamada para o WhatsApp.</t>
+          <t>Confirmar a disponibilidade antes de publicar.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="78" customHeight="1" s="16">
       <c r="A25" s="22" t="n">
-        <v>46374</v>
+        <v>46375</v>
       </c>
       <c r="B25" s="23">
         <f>TEXT(A25,"dddd")</f>
@@ -1902,32 +1902,32 @@
       </c>
       <c r="C25" s="23" t="inlineStr">
         <is>
-          <t>Google Perfil</t>
+          <t>Instagram</t>
         </is>
       </c>
       <c r="D25" s="23" t="inlineStr">
         <is>
-          <t>Post</t>
+          <t>Reels</t>
         </is>
       </c>
       <c r="E25" s="23" t="inlineStr">
         <is>
-          <t>Campanha</t>
+          <t>Depoimento</t>
         </is>
       </c>
       <c r="F25" s="23" t="inlineStr">
         <is>
-          <t>Réveillon: poucos quartos</t>
+          <t>Obrigado pelo ano</t>
         </is>
       </c>
       <c r="G25" s="23" t="inlineStr">
         <is>
-          <t>Quer começar o ano em paz? Restam poucos quartos para o Réveillon. Chame no WhatsApp.</t>
+          <t>O que mais ouvimos neste ano: atendimento de família e sossego. Obrigado por confiar na gente.</t>
         </is>
       </c>
       <c r="H25" s="23" t="inlineStr">
         <is>
-          <t>#VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+          <t>#Depoimento #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
         </is>
       </c>
       <c r="I25" s="23" t="inlineStr">
@@ -1942,13 +1942,13 @@
       </c>
       <c r="K25" s="23" t="inlineStr">
         <is>
-          <t>Confirmar a disponibilidade antes de publicar.</t>
+          <t>Só depoimentos autorizados.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="78" customHeight="1" s="16">
       <c r="A26" s="22" t="n">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="B26" s="23">
         <f>TEXT(A26,"dddd")</f>
@@ -1956,32 +1956,32 @@
       </c>
       <c r="C26" s="23" t="inlineStr">
         <is>
-          <t>Instagram</t>
+          <t>Facebook</t>
         </is>
       </c>
       <c r="D26" s="23" t="inlineStr">
         <is>
-          <t>Reels</t>
+          <t>Vídeo</t>
         </is>
       </c>
       <c r="E26" s="23" t="inlineStr">
         <is>
-          <t>Depoimento</t>
+          <t>Campanha</t>
         </is>
       </c>
       <c r="F26" s="23" t="inlineStr">
         <is>
-          <t>Obrigado pelo ano</t>
+          <t>Última chamada do Natal</t>
         </is>
       </c>
       <c r="G26" s="23" t="inlineStr">
         <is>
-          <t>O que mais ouvimos neste ano: atendimento de família e sossego. Obrigado por confiar na gente.</t>
+          <t>Ainda dá tempo de passar o Natal em Matilde. Chame no WhatsApp.</t>
         </is>
       </c>
       <c r="H26" s="23" t="inlineStr">
         <is>
-          <t>#Depoimento #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+          <t>#NatalEmMatilde #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
         </is>
       </c>
       <c r="I26" s="23" t="inlineStr">
@@ -1996,13 +1996,13 @@
       </c>
       <c r="K26" s="23" t="inlineStr">
         <is>
-          <t>Só depoimentos autorizados.</t>
+          <t>Publicar só se houver quartos livres.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="78" customHeight="1" s="16">
       <c r="A27" s="22" t="n">
-        <v>46379</v>
+        <v>46380</v>
       </c>
       <c r="B27" s="23">
         <f>TEXT(A27,"dddd")</f>
@@ -2010,32 +2010,32 @@
       </c>
       <c r="C27" s="23" t="inlineStr">
         <is>
-          <t>Facebook</t>
+          <t>Google Perfil</t>
         </is>
       </c>
       <c r="D27" s="23" t="inlineStr">
         <is>
-          <t>Vídeo</t>
+          <t>Post</t>
         </is>
       </c>
       <c r="E27" s="23" t="inlineStr">
         <is>
-          <t>Campanha</t>
+          <t>Depoimento</t>
         </is>
       </c>
       <c r="F27" s="23" t="inlineStr">
         <is>
-          <t>Última chamada do Natal</t>
+          <t>Obrigado pelas avaliações</t>
         </is>
       </c>
       <c r="G27" s="23" t="inlineStr">
         <is>
-          <t>Ainda dá tempo de passar o Natal em Matilde. Chame no WhatsApp.</t>
+          <t>Nota 4,7 no Google. Obrigado a quem já se hospedou com a gente. A sua avaliação ajuda outras pessoas a nos encontrar.</t>
         </is>
       </c>
       <c r="H27" s="23" t="inlineStr">
         <is>
-          <t>#NatalEmMatilde #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+          <t>#VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
         </is>
       </c>
       <c r="I27" s="23" t="inlineStr">
@@ -2050,13 +2050,13 @@
       </c>
       <c r="K27" s="23" t="inlineStr">
         <is>
-          <t>Publicar só se houver quartos livres.</t>
+          <t>Responder também às avaliações recentes.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="78" customHeight="1" s="16">
       <c r="A28" s="22" t="n">
-        <v>46384</v>
+        <v>46382</v>
       </c>
       <c r="B28" s="23">
         <f>TEXT(A28,"dddd")</f>
@@ -2110,7 +2110,7 @@
     </row>
     <row r="29" ht="78" customHeight="1" s="16">
       <c r="A29" s="22" t="n">
-        <v>46386</v>
+        <v>46384</v>
       </c>
       <c r="B29" s="23">
         <f>TEXT(A29,"dddd")</f>
@@ -2118,62 +2118,103 @@
       </c>
       <c r="C29" s="23" t="inlineStr">
         <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="D29" s="23" t="inlineStr">
+        <is>
+          <t>Vídeo</t>
+        </is>
+      </c>
+      <c r="E29" s="23" t="inlineStr">
+        <is>
+          <t>Experiência</t>
+        </is>
+      </c>
+      <c r="F29" s="23" t="inlineStr">
+        <is>
+          <t>A rede diante das orquídeas</t>
+        </is>
+      </c>
+      <c r="G29" s="23" t="inlineStr">
+        <is>
+          <t>Cada quarto tem uma rede para balançar diante das orquídeas. Aqui o sossego tem lugar marcado.</t>
+        </is>
+      </c>
+      <c r="H29" s="23" t="inlineStr">
+        <is>
+          <t>#Sossego #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
+        </is>
+      </c>
+      <c r="I29" s="23" t="inlineStr">
+        <is>
+          <t>Dono</t>
+        </is>
+      </c>
+      <c r="J29" s="26" t="inlineStr">
+        <is>
+          <t>Ideia</t>
+        </is>
+      </c>
+      <c r="K29" s="23" t="inlineStr">
+        <is>
+          <t>Plano aberto da rede, sem corte rápido, com som ambiente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="78" customHeight="1" s="16">
+      <c r="A30" s="22" t="n">
+        <v>46387</v>
+      </c>
+      <c r="B30" s="23">
+        <f>TEXT(A30,"dddd")</f>
+        <v/>
+      </c>
+      <c r="C30" s="23" t="inlineStr">
+        <is>
           <t>Instagram</t>
         </is>
       </c>
-      <c r="D29" s="23" t="inlineStr">
+      <c r="D30" s="23" t="inlineStr">
         <is>
           <t>Reels</t>
         </is>
       </c>
-      <c r="E29" s="23" t="inlineStr">
+      <c r="E30" s="23" t="inlineStr">
         <is>
           <t>Campanha</t>
         </is>
       </c>
-      <c r="F29" s="23" t="inlineStr">
+      <c r="F30" s="23" t="inlineStr">
         <is>
           <t>Boas festas e feliz 2027</t>
         </is>
       </c>
-      <c r="G29" s="23" t="inlineStr">
+      <c r="G30" s="23" t="inlineStr">
         <is>
           <t>Que 2027 comece com sossego. Feliz Ano Novo de toda a Vila Mathilde.</t>
         </is>
       </c>
-      <c r="H29" s="23" t="inlineStr">
+      <c r="H30" s="23" t="inlineStr">
         <is>
           <t>#FelizAnoNovo #VilaMathilde #Matilde #AlfredoChaves #MontanhasCapixabas</t>
         </is>
       </c>
-      <c r="I29" s="23" t="inlineStr">
+      <c r="I30" s="23" t="inlineStr">
         <is>
           <t>Dono</t>
         </is>
       </c>
-      <c r="J29" s="26" t="inlineStr">
+      <c r="J30" s="26" t="inlineStr">
         <is>
           <t>Ideia</t>
         </is>
       </c>
-      <c r="K29" s="23" t="inlineStr">
+      <c r="K30" s="23" t="inlineStr">
         <is>
           <t>Vídeo de encerramento do ano.</t>
         </is>
       </c>
-    </row>
-    <row r="30" s="16">
-      <c r="A30" s="22" t="n"/>
-      <c r="B30" s="23" t="n"/>
-      <c r="C30" s="23" t="n"/>
-      <c r="D30" s="23" t="n"/>
-      <c r="E30" s="23" t="n"/>
-      <c r="F30" s="23" t="n"/>
-      <c r="G30" s="23" t="n"/>
-      <c r="H30" s="23" t="n"/>
-      <c r="I30" s="23" t="n"/>
-      <c r="J30" s="23" t="n"/>
-      <c r="K30" s="23" t="n"/>
     </row>
     <row r="31" s="16">
       <c r="A31" s="22" t="n"/>

</xml_diff>